<commit_message>
Dice faces shown as stacked opposite pairs (6/1, 5/2, 4/3) with a ↕ arrow
Relic strip + install panel now stack each opposite pair vertically with a
double-headed arrow, so the Heavy/Weighted pairing is obvious. Also recorded
the 12 permanent rule-unlocks in the design catalog.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DESIGN/craps-roguelike-catalog.xlsx
+++ b/DESIGN/craps-roguelike-catalog.xlsx
@@ -2152,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2416,6 +2416,364 @@
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>- Currency is Markers, earned by clearing rounds (+ leftover-bullet bonus, + Interest relic).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>PERMANENT RULE UNLOCKS (Table Access - purchased, added to the felt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Unlock</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Prerequisite</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Double Odds</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Odds</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>2x odds on Pass / Come / Don'ts</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>engine ready; needs odds-placement UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Table Odds</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Odds</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>3x/4x/5x odds (3x on 4 &amp; 10, 4x on 5 &amp; 9, 5x on 6 &amp; 8)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Double Odds</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>engine ready; needs odds UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Five Times Odds</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Odds</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>5x odds on all points</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Table Odds</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>engine ready; needs odds UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Hard Four</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Hardway</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Hard Four bet</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Hard Six</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Hardway</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Hard Six bet</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Hard Eight</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Hardway</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Hard Eight bet</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Hard Ten</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Hardway</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Hard Ten bet</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Big Red</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Any Seven bet</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Craps</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Any Craps bet</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Horn Bet</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the Horn bet + the hopping 2, 12, 3, 11</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs felt + hop spots</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Hardway Hops</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Unlock the hop bets for 22, 33, 44, 55</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs hop grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Hop Bets</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Unlock all the 16-for-1 hop bets</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>resolver-ready; needs hop grid</t>
         </is>
       </c>
     </row>

</xml_diff>